<commit_message>
Descripción Descarga de centralizadores hasta 3ro SEC
</commit_message>
<xml_diff>
--- a/public/templates/CenBth3.xlsx
+++ b/public/templates/CenBth3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Gestion2025\Notas 2025\2doTRIM\BTH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\saat\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D9497B-9F50-4524-988A-5E54EF3D9C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26DE5712-3F2C-44DE-A0C5-E4B7B644E6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
   <si>
     <t>Nº</t>
   </si>
@@ -76,10 +76,7 @@
 BTH</t>
   </si>
   <si>
-    <t>T3</t>
-  </si>
-  <si>
-    <t>GESTIÓN 2025 NOTAS OFICIALES 1ER TRIMESTRE</t>
+    <t>GESTIÓN 2026 NOTAS OFICIALES 1ER TRIMESTRE</t>
   </si>
 </sst>
 </file>
@@ -92,7 +89,7 @@
     <numFmt numFmtId="166" formatCode="#.00"/>
     <numFmt numFmtId="167" formatCode="%#.00"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -303,6 +300,14 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1029,7 +1034,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1045,9 +1050,6 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1115,9 +1117,6 @@
     <xf numFmtId="0" fontId="29" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="1" fontId="28" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1230,6 +1229,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1747,72 +1755,72 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B4" s="50" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
+      <c r="B4" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="51"/>
-      <c r="I5" s="51"/>
-      <c r="J5" s="51"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
     </row>
     <row r="6" spans="1:17" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="54" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="56" t="s">
+      <c r="B6" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="58"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="61"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="33" t="s">
+      <c r="D6" s="56"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="59"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="70" t="s">
         <v>12</v>
       </c>
       <c r="K6" s="1"/>
@@ -1824,9 +1832,9 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="63"/>
-      <c r="B7" s="55"/>
-      <c r="C7" s="57"/>
+      <c r="A7" s="61"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="55"/>
       <c r="D7" s="4" t="s">
         <v>8</v>
       </c>
@@ -1845,686 +1853,684 @@
       <c r="I7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="71"/>
+    </row>
+    <row r="8" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14"/>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="14">
+        <f>E8+G8+I8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="14"/>
+      <c r="B9" s="15">
+        <v>2</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="14">
+        <f t="shared" ref="J9:J37" si="0">E9+G9+I9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14"/>
+      <c r="B10" s="15">
+        <v>3</v>
+      </c>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="14"/>
+      <c r="B11" s="15">
+        <v>4</v>
+      </c>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="15">
+        <v>5</v>
+      </c>
+      <c r="C12" s="16"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22"/>
+      <c r="B13" s="15">
+        <v>6</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="72"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="14"/>
+      <c r="B14" s="15">
+        <v>7</v>
+      </c>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="15">
+        <v>8</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="15">
+        <v>9</v>
+      </c>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15">
+        <v>10</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22"/>
+      <c r="B18" s="15">
+        <v>11</v>
+      </c>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="15">
+        <v>12</v>
+      </c>
+      <c r="C19" s="16"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14"/>
+      <c r="B20" s="15">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="8">
-        <v>1</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="15">
-        <f>E8+G8+I8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="16">
-        <v>2</v>
-      </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="15">
-        <f t="shared" ref="J9:J37" si="0">E9+G9+I9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="16">
+      <c r="C20" s="16"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14"/>
+      <c r="B21" s="15">
+        <v>14</v>
+      </c>
+      <c r="C21" s="16"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="14"/>
+      <c r="B22" s="15">
+        <v>15</v>
+      </c>
+      <c r="C22" s="16"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="22"/>
+      <c r="B23" s="15">
+        <v>16</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="14"/>
+      <c r="B24" s="15">
+        <v>17</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14"/>
+      <c r="B25" s="15">
+        <v>18</v>
+      </c>
+      <c r="C25" s="16"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="14"/>
+      <c r="B26" s="15">
+        <v>19</v>
+      </c>
+      <c r="C26" s="23"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="14"/>
+      <c r="B27" s="15">
+        <v>20</v>
+      </c>
+      <c r="C27" s="16"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22"/>
+      <c r="B28" s="15">
+        <v>21</v>
+      </c>
+      <c r="C28" s="16"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="14"/>
+      <c r="B29" s="15">
+        <v>22</v>
+      </c>
+      <c r="C29" s="16"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="14"/>
+      <c r="B30" s="15">
+        <v>23</v>
+      </c>
+      <c r="C30" s="16"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="14"/>
+      <c r="B31" s="15">
+        <v>24</v>
+      </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="14"/>
+      <c r="B32" s="15">
+        <v>25</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="22"/>
+      <c r="B33" s="15">
+        <v>26</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="14"/>
+      <c r="B34" s="15">
+        <v>27</v>
+      </c>
+      <c r="C34" s="16"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="19"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="14"/>
+      <c r="B35" s="15">
+        <v>28</v>
+      </c>
+      <c r="C35" s="16"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="14"/>
+      <c r="B36" s="15">
+        <v>29</v>
+      </c>
+      <c r="C36" s="16"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="19"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="31"/>
+      <c r="B37" s="24">
+        <v>30</v>
+      </c>
+      <c r="C37" s="25"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="31">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="16">
+      <c r="C38" s="65"/>
+      <c r="D38" s="32" t="str">
+        <f>IF(SUM(D8:D37)=0,"",AVERAGE(D8:D37))</f>
+        <v/>
+      </c>
+      <c r="E38" s="33" t="str">
+        <f t="shared" ref="E38:J38" si="1">IF(SUM(E8:E37)=0,"",AVERAGE(E8:E37))</f>
+        <v/>
+      </c>
+      <c r="F38" s="34" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="G38" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="H38" s="36" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I38" s="37" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J38" s="38" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="66" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="16">
+      <c r="C39" s="67"/>
+      <c r="D39" s="32" t="str">
+        <f>IF(SUM(D8:D37)=0,"",MEDIAN(D8:D37))</f>
+        <v/>
+      </c>
+      <c r="E39" s="33" t="str">
+        <f t="shared" ref="E39:J39" si="2">IF(SUM(E8:E37)=0,"",MEDIAN(E8:E37))</f>
+        <v/>
+      </c>
+      <c r="F39" s="34" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="G39" s="35" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H39" s="36" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I39" s="37" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="J39" s="38" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="23"/>
-      <c r="B13" s="16">
+      <c r="C40" s="67"/>
+      <c r="D40" s="32" t="str">
+        <f>IF(SUM(D8:D37)=0,"",MAX(D8:D37))</f>
+        <v/>
+      </c>
+      <c r="E40" s="33" t="str">
+        <f t="shared" ref="E40:J40" si="3">IF(SUM(E8:E37)=0,"",MAX(E8:E37))</f>
+        <v/>
+      </c>
+      <c r="F40" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="G40" s="35" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="H40" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="I40" s="37" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="J40" s="38" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16">
+      <c r="C41" s="67"/>
+      <c r="D41" s="32" t="str">
+        <f>IF(SUM(D8:D37)=0,"",MIN(D8:D37))</f>
+        <v/>
+      </c>
+      <c r="E41" s="33" t="str">
+        <f t="shared" ref="E41:J41" si="4">IF(SUM(E8:E37)=0,"",MIN(E8:E37))</f>
+        <v/>
+      </c>
+      <c r="F41" s="34" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G41" s="35" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="H41" s="36" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="I41" s="37" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="J41" s="38" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16">
-        <v>8</v>
-      </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16">
-        <v>9</v>
-      </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16">
-        <v>10</v>
-      </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="23"/>
-      <c r="B18" s="16">
-        <v>11</v>
-      </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16">
-        <v>12</v>
-      </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16">
-        <v>13</v>
-      </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="15"/>
-      <c r="B21" s="16">
-        <v>14</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="16">
-        <v>15</v>
-      </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="23"/>
-      <c r="B23" s="16">
-        <v>16</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="16">
-        <v>17</v>
-      </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
-      <c r="B25" s="16">
-        <v>18</v>
-      </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="16">
-        <v>19</v>
-      </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="22"/>
-      <c r="J26" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="16">
-        <v>20</v>
-      </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="23"/>
-      <c r="B28" s="16">
-        <v>21</v>
-      </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="16">
-        <v>22</v>
-      </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
-      <c r="B30" s="16">
-        <v>23</v>
-      </c>
-      <c r="C30" s="17"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="15"/>
-      <c r="B31" s="16">
-        <v>24</v>
-      </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="22"/>
-      <c r="J31" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="15"/>
-      <c r="B32" s="16">
-        <v>25</v>
-      </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="23"/>
-      <c r="B33" s="16">
-        <v>26</v>
-      </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16">
-        <v>27</v>
-      </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="15"/>
-      <c r="B35" s="16">
-        <v>28</v>
-      </c>
-      <c r="C35" s="17"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="21"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
-      <c r="B36" s="16">
-        <v>29</v>
-      </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="32"/>
-      <c r="B37" s="25">
-        <v>30</v>
-      </c>
-      <c r="C37" s="26"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="28"/>
-      <c r="F37" s="29"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="29"/>
-      <c r="I37" s="31"/>
-      <c r="J37" s="32">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="66" t="s">
-        <v>3</v>
-      </c>
-      <c r="C38" s="67"/>
-      <c r="D38" s="34" t="str">
-        <f>IF(SUM(D8:D37)=0,"",AVERAGE(D8:D37))</f>
-        <v/>
-      </c>
-      <c r="E38" s="35" t="str">
-        <f t="shared" ref="E38:J38" si="1">IF(SUM(E8:E37)=0,"",AVERAGE(E8:E37))</f>
-        <v/>
-      </c>
-      <c r="F38" s="36" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="G38" s="37" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="H38" s="38" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I38" s="39" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J38" s="40" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="68" t="s">
-        <v>4</v>
-      </c>
-      <c r="C39" s="69"/>
-      <c r="D39" s="34" t="str">
-        <f>IF(SUM(D8:D37)=0,"",MEDIAN(D8:D37))</f>
-        <v/>
-      </c>
-      <c r="E39" s="35" t="str">
-        <f t="shared" ref="E39:J39" si="2">IF(SUM(E8:E37)=0,"",MEDIAN(E8:E37))</f>
-        <v/>
-      </c>
-      <c r="F39" s="36" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="G39" s="37" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="H39" s="38" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="I39" s="39" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J39" s="40" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="68" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" s="69"/>
-      <c r="D40" s="34" t="str">
-        <f>IF(SUM(D8:D37)=0,"",MAX(D8:D37))</f>
-        <v/>
-      </c>
-      <c r="E40" s="35" t="str">
-        <f t="shared" ref="E40:J40" si="3">IF(SUM(E8:E37)=0,"",MAX(E8:E37))</f>
-        <v/>
-      </c>
-      <c r="F40" s="36" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="G40" s="37" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="H40" s="38" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="I40" s="39" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J40" s="40" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="68" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="69"/>
-      <c r="D41" s="34" t="str">
-        <f>IF(SUM(D8:D37)=0,"",MIN(D8:D37))</f>
-        <v/>
-      </c>
-      <c r="E41" s="35" t="str">
-        <f t="shared" ref="E41:J41" si="4">IF(SUM(E8:E37)=0,"",MIN(E8:E37))</f>
-        <v/>
-      </c>
-      <c r="F41" s="36" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="G41" s="37" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="H41" s="38" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="I41" s="39" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J41" s="40" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="70" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="71"/>
-      <c r="D42" s="41" t="str">
+      <c r="C42" s="69"/>
+      <c r="D42" s="39" t="str">
         <f>IF(D38="","",COUNTIF(D8:D37,"&lt;51")/COUNT(D8:D37)*100)</f>
         <v/>
       </c>
-      <c r="E42" s="42" t="str">
+      <c r="E42" s="40" t="str">
         <f t="shared" ref="E42:J42" si="5">IF(E38="","",COUNTIF(E8:E37,"&lt;51")/COUNT(E8:E37)*100)</f>
         <v/>
       </c>
-      <c r="F42" s="43" t="str">
+      <c r="F42" s="41" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="G42" s="44" t="str">
+      <c r="G42" s="42" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="H42" s="45" t="str">
+      <c r="H42" s="43" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="I42" s="46" t="str">
+      <c r="I42" s="44" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J42" s="47" t="str">
+      <c r="J42" s="45" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -2607,21 +2613,21 @@
       <c r="J49" s="5"/>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="E51" s="64"/>
-      <c r="F51" s="65"/>
-      <c r="G51" s="65"/>
-      <c r="H51" s="65"/>
-      <c r="I51" s="65"/>
+      <c r="E51" s="62"/>
+      <c r="F51" s="63"/>
+      <c r="G51" s="63"/>
+      <c r="H51" s="63"/>
+      <c r="I51" s="63"/>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="E52" s="65"/>
-      <c r="F52" s="65"/>
-      <c r="G52" s="65"/>
-      <c r="H52" s="65"/>
-      <c r="I52" s="65"/>
+      <c r="E52" s="63"/>
+      <c r="F52" s="63"/>
+      <c r="G52" s="63"/>
+      <c r="H52" s="63"/>
+      <c r="I52" s="63"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="E51:I51"/>
     <mergeCell ref="E52:I52"/>
@@ -2639,6 +2645,7 @@
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="J6:J7"/>
   </mergeCells>
   <conditionalFormatting sqref="J8:J37">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
@@ -2647,7 +2654,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.57604166666666667" right="0.25" top="0.21875" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="79" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup scale="77" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>